<commit_message>
ajout nouveau cv annonyme
</commit_message>
<xml_diff>
--- a/Tableau/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthe_se.xlsx
+++ b/Tableau/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthe_se.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portefolio\Tableau\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Portefolio\KindnesSoul.github.io\Tableau\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9CC1DB53-D337-4F80-98B5-A5A710B831E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF85ABA1-1756-452A-9D7B-FFD3BE749557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$48</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="48">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -138,6 +138,54 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>2 ème Stage</t>
+  </si>
+  <si>
+    <t>30/01/25 à 22/05/25</t>
+  </si>
+  <si>
+    <t>Suivi le cahier des charges imposer de l'hypothétique client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ce conformer au regle RGPD </t>
+  </si>
+  <si>
+    <t>Participation à la valorisation en ligne de l'image de l'organisation GranR via un site web sur Wordpress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en place d'un guide d'utilisation et d'installation du service </t>
+  </si>
+  <si>
+    <t>Mise en plan d'un environnement d'apprentissage personnel pour apprendre le FrameWork NestJS ainsi que le NodeJS et le TypeScript</t>
+  </si>
+  <si>
+    <t>Réalisations Personnel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planification et partage des taches entre diférents collaborateur </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planification et partage des taches entre diférents developpeur </t>
+  </si>
+  <si>
+    <t>AP3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mise en palce et creation d'une base de donnée / different niveau d'habilitation entre utilisateur et admin </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service déployer sur un serveur accecible via le résau de mon etablissement  / Mise en place d'un guide d'utilisation et d'installation du service </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suivi le cahier du cahier des charges imposer par ma tutrice de stage </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Organisation personnel vis-à-vis du poc (Proof of concept) qui ma étais demander </t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai déployer mon poc en serveur dev ou j'ai pu tester et reussir les api de connexion entre mon poc Back end et le front de leur application </t>
   </si>
 </sst>
 </file>
@@ -210,15 +258,27 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -604,12 +664,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -617,13 +690,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -632,22 +705,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -656,29 +723,101 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -703,60 +842,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1066,94 +1151,94 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AQ94"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.85546875" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="23"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="H1" s="37"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
+      <c r="B2" s="37"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="30" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="31"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="53"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="14" t="s">
+      <c r="B4" s="50"/>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="42" t="s">
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="44"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="32" t="s">
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="41" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1175,25 +1260,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="41"/>
-      <c r="C7" s="46" t="s">
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="36"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="46" t="s">
+      <c r="E7" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="46" t="s">
+      <c r="F7" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="46" t="s">
+      <c r="G7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="48" t="s">
+      <c r="H7" s="22" t="s">
         <v>14</v>
       </c>
       <c r="I7"/>
@@ -1232,17 +1317,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="34" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="36"/>
+      <c r="B8" s="39"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="39"/>
+      <c r="F8" s="39"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="40"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1279,29 +1364,29 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="47" t="s">
+      <c r="D9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="47" t="s">
+      <c r="E9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="47" t="s">
+      <c r="F9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="G9" s="47" t="s">
+      <c r="G9" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="17"/>
+      <c r="H9" s="15"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1338,15 +1423,17 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="10"/>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>35</v>
+      </c>
       <c r="B10" s="8"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="15"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1383,27 +1470,17 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
-        <v>28</v>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>34</v>
       </c>
       <c r="B11" s="8"/>
-      <c r="C11" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="G11" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="H11" s="17"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="15"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1440,15 +1517,17 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>36</v>
+      </c>
       <c r="B12" s="8"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="17"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="15"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1485,15 +1564,17 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>40</v>
+      </c>
       <c r="B13" s="8"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="17"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="15"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1530,15 +1611,17 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>37</v>
+      </c>
       <c r="B14" s="8"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="17"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="15"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1575,15 +1658,15 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
       <c r="B15" s="8"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="17"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="15"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1620,15 +1703,29 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="17"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H16" s="15"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1665,15 +1762,17 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="10"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>43</v>
+      </c>
       <c r="B17" s="8"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="17"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="15"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1710,15 +1809,17 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="B18" s="8"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="17"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="15"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1755,17 +1856,15 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="39"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="15"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1802,27 +1901,17 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
-        <v>29</v>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="9" t="s">
+        <v>41</v>
       </c>
       <c r="B20" s="8"/>
-      <c r="C20" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="D20" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="E20" s="16"/>
-      <c r="F20" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="G20" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="H20" s="49" t="s">
-        <v>31</v>
-      </c>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="15"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1859,15 +1948,17 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
+        <v>37</v>
+      </c>
       <c r="B21" s="8"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="17"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="15"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1904,15 +1995,15 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
       <c r="B22" s="8"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="17"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="15"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1949,15 +2040,25 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10"/>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>42</v>
+      </c>
       <c r="B23" s="8"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="17"/>
+      <c r="C23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H23" s="15"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1994,15 +2095,17 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="10"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>43</v>
+      </c>
       <c r="B24" s="8"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="17"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="15"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2039,15 +2142,17 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="9" t="s">
+        <v>34</v>
+      </c>
       <c r="B25" s="8"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="17"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="15"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2084,15 +2189,15 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10"/>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
       <c r="B26" s="8"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="17"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="15"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2129,17 +2234,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="37" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="38"/>
-      <c r="C27" s="38"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="39"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="8"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="26"/>
+      <c r="H27" s="15"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2176,15 +2281,17 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>44</v>
+      </c>
       <c r="B28" s="8"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="17"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="15"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2221,15 +2328,14 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="10"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="8"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="17"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="26"/>
+      <c r="H29" s="15"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2266,15 +2372,17 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="10"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="17"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A30" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="33"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="34"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2311,15 +2419,27 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="10"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="B31" s="8"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="17"/>
+      <c r="C31" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31" s="14"/>
+      <c r="F31" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="H31" s="23" t="s">
+        <v>31</v>
+      </c>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2356,15 +2476,15 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="10"/>
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
       <c r="B32" s="8"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="17"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="15"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2401,15 +2521,17 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="9"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="19"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B33" s="8"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="15"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2446,15 +2568,14 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="21"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="15"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2491,15 +2612,17 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" s="8"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="15"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2536,66 +2659,662 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="8"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="15"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+      <c r="S36"/>
+      <c r="T36"/>
+      <c r="U36"/>
+      <c r="V36"/>
+      <c r="W36"/>
+      <c r="X36"/>
+      <c r="Y36"/>
+      <c r="Z36"/>
+      <c r="AA36"/>
+      <c r="AB36"/>
+      <c r="AC36"/>
+      <c r="AD36"/>
+      <c r="AE36"/>
+      <c r="AF36"/>
+      <c r="AG36"/>
+      <c r="AH36"/>
+      <c r="AI36"/>
+      <c r="AJ36"/>
+      <c r="AK36"/>
+      <c r="AL36"/>
+      <c r="AM36"/>
+      <c r="AN36"/>
+      <c r="AO36"/>
+      <c r="AP36"/>
+      <c r="AQ36"/>
+    </row>
+    <row r="37" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" s="8"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="27"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37"/>
+      <c r="P37"/>
+      <c r="Q37"/>
+      <c r="R37"/>
+      <c r="S37"/>
+      <c r="T37"/>
+      <c r="U37"/>
+      <c r="V37"/>
+      <c r="W37"/>
+      <c r="X37"/>
+      <c r="Y37"/>
+      <c r="Z37"/>
+      <c r="AA37"/>
+      <c r="AB37"/>
+      <c r="AC37"/>
+      <c r="AD37"/>
+      <c r="AE37"/>
+      <c r="AF37"/>
+      <c r="AG37"/>
+      <c r="AH37"/>
+      <c r="AI37"/>
+      <c r="AJ37"/>
+      <c r="AK37"/>
+      <c r="AL37"/>
+      <c r="AM37"/>
+      <c r="AN37"/>
+      <c r="AO37"/>
+      <c r="AP37"/>
+      <c r="AQ37"/>
+    </row>
+    <row r="38" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A38" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="33"/>
+      <c r="D38" s="33"/>
+      <c r="E38" s="33"/>
+      <c r="F38" s="33"/>
+      <c r="G38" s="33"/>
+      <c r="H38" s="34"/>
+      <c r="I38"/>
+      <c r="J38"/>
+      <c r="K38"/>
+      <c r="L38"/>
+      <c r="M38"/>
+      <c r="N38"/>
+      <c r="O38"/>
+      <c r="P38"/>
+      <c r="Q38"/>
+      <c r="R38"/>
+      <c r="S38"/>
+      <c r="T38"/>
+      <c r="U38"/>
+      <c r="V38"/>
+      <c r="W38"/>
+      <c r="X38"/>
+      <c r="Y38"/>
+      <c r="Z38"/>
+      <c r="AA38"/>
+      <c r="AB38"/>
+      <c r="AC38"/>
+      <c r="AD38"/>
+      <c r="AE38"/>
+      <c r="AF38"/>
+      <c r="AG38"/>
+      <c r="AH38"/>
+      <c r="AI38"/>
+      <c r="AJ38"/>
+      <c r="AK38"/>
+      <c r="AL38"/>
+      <c r="AM38"/>
+      <c r="AN38"/>
+      <c r="AO38"/>
+      <c r="AP38"/>
+      <c r="AQ38"/>
+    </row>
+    <row r="39" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B39" s="8"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="15"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+      <c r="L39"/>
+      <c r="M39"/>
+      <c r="N39"/>
+      <c r="O39"/>
+      <c r="P39"/>
+      <c r="Q39"/>
+      <c r="R39"/>
+      <c r="S39"/>
+      <c r="T39"/>
+      <c r="U39"/>
+      <c r="V39"/>
+      <c r="W39"/>
+      <c r="X39"/>
+      <c r="Y39"/>
+      <c r="Z39"/>
+      <c r="AA39"/>
+      <c r="AB39"/>
+      <c r="AC39"/>
+      <c r="AD39"/>
+      <c r="AE39"/>
+      <c r="AF39"/>
+      <c r="AG39"/>
+      <c r="AH39"/>
+      <c r="AI39"/>
+      <c r="AJ39"/>
+      <c r="AK39"/>
+      <c r="AL39"/>
+      <c r="AM39"/>
+      <c r="AN39"/>
+      <c r="AO39"/>
+      <c r="AP39"/>
+      <c r="AQ39"/>
+    </row>
+    <row r="40" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="9"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="15"/>
+      <c r="I40"/>
+      <c r="J40"/>
+      <c r="K40"/>
+      <c r="L40"/>
+      <c r="M40"/>
+      <c r="N40"/>
+      <c r="O40"/>
+      <c r="P40"/>
+      <c r="Q40"/>
+      <c r="R40"/>
+      <c r="S40"/>
+      <c r="T40"/>
+      <c r="U40"/>
+      <c r="V40"/>
+      <c r="W40"/>
+      <c r="X40"/>
+      <c r="Y40"/>
+      <c r="Z40"/>
+      <c r="AA40"/>
+      <c r="AB40"/>
+      <c r="AC40"/>
+      <c r="AD40"/>
+      <c r="AE40"/>
+      <c r="AF40"/>
+      <c r="AG40"/>
+      <c r="AH40"/>
+      <c r="AI40"/>
+      <c r="AJ40"/>
+      <c r="AK40"/>
+      <c r="AL40"/>
+      <c r="AM40"/>
+      <c r="AN40"/>
+      <c r="AO40"/>
+      <c r="AP40"/>
+      <c r="AQ40"/>
+    </row>
+    <row r="41" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="9"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="15"/>
+      <c r="I41"/>
+      <c r="J41"/>
+      <c r="K41"/>
+      <c r="L41"/>
+      <c r="M41"/>
+      <c r="N41"/>
+      <c r="O41"/>
+      <c r="P41"/>
+      <c r="Q41"/>
+      <c r="R41"/>
+      <c r="S41"/>
+      <c r="T41"/>
+      <c r="U41"/>
+      <c r="V41"/>
+      <c r="W41"/>
+      <c r="X41"/>
+      <c r="Y41"/>
+      <c r="Z41"/>
+      <c r="AA41"/>
+      <c r="AB41"/>
+      <c r="AC41"/>
+      <c r="AD41"/>
+      <c r="AE41"/>
+      <c r="AF41"/>
+      <c r="AG41"/>
+      <c r="AH41"/>
+      <c r="AI41"/>
+      <c r="AJ41"/>
+      <c r="AK41"/>
+      <c r="AL41"/>
+      <c r="AM41"/>
+      <c r="AN41"/>
+      <c r="AO41"/>
+      <c r="AP41"/>
+      <c r="AQ41"/>
+    </row>
+    <row r="42" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="9"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="15"/>
+      <c r="I42"/>
+      <c r="J42"/>
+      <c r="K42"/>
+      <c r="L42"/>
+      <c r="M42"/>
+      <c r="N42"/>
+      <c r="O42"/>
+      <c r="P42"/>
+      <c r="Q42"/>
+      <c r="R42"/>
+      <c r="S42"/>
+      <c r="T42"/>
+      <c r="U42"/>
+      <c r="V42"/>
+      <c r="W42"/>
+      <c r="X42"/>
+      <c r="Y42"/>
+      <c r="Z42"/>
+      <c r="AA42"/>
+      <c r="AB42"/>
+      <c r="AC42"/>
+      <c r="AD42"/>
+      <c r="AE42"/>
+      <c r="AF42"/>
+      <c r="AG42"/>
+      <c r="AH42"/>
+      <c r="AI42"/>
+      <c r="AJ42"/>
+      <c r="AK42"/>
+      <c r="AL42"/>
+      <c r="AM42"/>
+      <c r="AN42"/>
+      <c r="AO42"/>
+      <c r="AP42"/>
+      <c r="AQ42"/>
+    </row>
+    <row r="43" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="9"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="15"/>
+      <c r="I43"/>
+      <c r="J43"/>
+      <c r="K43"/>
+      <c r="L43"/>
+      <c r="M43"/>
+      <c r="N43"/>
+      <c r="O43"/>
+      <c r="P43"/>
+      <c r="Q43"/>
+      <c r="R43"/>
+      <c r="S43"/>
+      <c r="T43"/>
+      <c r="U43"/>
+      <c r="V43"/>
+      <c r="W43"/>
+      <c r="X43"/>
+      <c r="Y43"/>
+      <c r="Z43"/>
+      <c r="AA43"/>
+      <c r="AB43"/>
+      <c r="AC43"/>
+      <c r="AD43"/>
+      <c r="AE43"/>
+      <c r="AF43"/>
+      <c r="AG43"/>
+      <c r="AH43"/>
+      <c r="AI43"/>
+      <c r="AJ43"/>
+      <c r="AK43"/>
+      <c r="AL43"/>
+      <c r="AM43"/>
+      <c r="AN43"/>
+      <c r="AO43"/>
+      <c r="AP43"/>
+      <c r="AQ43"/>
+    </row>
+    <row r="44" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="15"/>
+      <c r="I44"/>
+      <c r="J44"/>
+      <c r="K44"/>
+      <c r="L44"/>
+      <c r="M44"/>
+      <c r="N44"/>
+      <c r="O44"/>
+      <c r="P44"/>
+      <c r="Q44"/>
+      <c r="R44"/>
+      <c r="S44"/>
+      <c r="T44"/>
+      <c r="U44"/>
+      <c r="V44"/>
+      <c r="W44"/>
+      <c r="X44"/>
+      <c r="Y44"/>
+      <c r="Z44"/>
+      <c r="AA44"/>
+      <c r="AB44"/>
+      <c r="AC44"/>
+      <c r="AD44"/>
+      <c r="AE44"/>
+      <c r="AF44"/>
+      <c r="AG44"/>
+      <c r="AH44"/>
+      <c r="AI44"/>
+      <c r="AJ44"/>
+      <c r="AK44"/>
+      <c r="AL44"/>
+      <c r="AM44"/>
+      <c r="AN44"/>
+      <c r="AO44"/>
+      <c r="AP44"/>
+      <c r="AQ44"/>
+    </row>
+    <row r="45" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="28"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
+      <c r="D45" s="30"/>
+      <c r="E45" s="30"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="30"/>
+      <c r="H45" s="31"/>
+      <c r="I45"/>
+      <c r="J45"/>
+      <c r="K45"/>
+      <c r="L45"/>
+      <c r="M45"/>
+      <c r="N45"/>
+      <c r="O45"/>
+      <c r="P45"/>
+      <c r="Q45"/>
+      <c r="R45"/>
+      <c r="S45"/>
+      <c r="T45"/>
+      <c r="U45"/>
+      <c r="V45"/>
+      <c r="W45"/>
+      <c r="X45"/>
+      <c r="Y45"/>
+      <c r="Z45"/>
+      <c r="AA45"/>
+      <c r="AB45"/>
+      <c r="AC45"/>
+      <c r="AD45"/>
+      <c r="AE45"/>
+      <c r="AF45"/>
+      <c r="AG45"/>
+      <c r="AH45"/>
+      <c r="AI45"/>
+      <c r="AJ45"/>
+      <c r="AK45"/>
+      <c r="AL45"/>
+      <c r="AM45"/>
+      <c r="AN45"/>
+      <c r="AO45"/>
+      <c r="AP45"/>
+      <c r="AQ45"/>
+    </row>
+    <row r="46" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A46" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="33"/>
+      <c r="F46" s="33"/>
+      <c r="G46" s="33"/>
+      <c r="H46" s="34"/>
+      <c r="I46"/>
+      <c r="J46"/>
+      <c r="K46"/>
+      <c r="L46"/>
+      <c r="M46"/>
+      <c r="N46"/>
+      <c r="O46"/>
+      <c r="P46"/>
+      <c r="Q46"/>
+      <c r="R46"/>
+      <c r="S46"/>
+      <c r="T46"/>
+      <c r="U46"/>
+      <c r="V46"/>
+      <c r="W46"/>
+      <c r="X46"/>
+      <c r="Y46"/>
+      <c r="Z46"/>
+      <c r="AA46"/>
+      <c r="AB46"/>
+      <c r="AC46"/>
+      <c r="AD46"/>
+      <c r="AE46"/>
+      <c r="AF46"/>
+      <c r="AG46"/>
+      <c r="AH46"/>
+      <c r="AI46"/>
+      <c r="AJ46"/>
+      <c r="AK46"/>
+      <c r="AL46"/>
+      <c r="AM46"/>
+      <c r="AN46"/>
+      <c r="AO46"/>
+      <c r="AP46"/>
+      <c r="AQ46"/>
+    </row>
+    <row r="47" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="10"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="16"/>
+      <c r="G47" s="16"/>
+      <c r="H47" s="17"/>
+      <c r="I47"/>
+      <c r="J47"/>
+      <c r="K47"/>
+      <c r="L47"/>
+      <c r="M47"/>
+      <c r="N47"/>
+      <c r="O47"/>
+      <c r="P47"/>
+      <c r="Q47"/>
+      <c r="R47"/>
+      <c r="S47"/>
+      <c r="T47"/>
+      <c r="U47"/>
+      <c r="V47"/>
+      <c r="W47"/>
+      <c r="X47"/>
+      <c r="Y47"/>
+      <c r="Z47"/>
+      <c r="AA47"/>
+      <c r="AB47"/>
+      <c r="AC47"/>
+      <c r="AD47"/>
+      <c r="AE47"/>
+      <c r="AF47"/>
+      <c r="AG47"/>
+      <c r="AH47"/>
+      <c r="AI47"/>
+      <c r="AJ47"/>
+      <c r="AK47"/>
+      <c r="AL47"/>
+      <c r="AM47"/>
+      <c r="AN47"/>
+      <c r="AO47"/>
+      <c r="AP47"/>
+      <c r="AQ47"/>
+    </row>
+    <row r="48" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A48" s="5"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48"/>
+      <c r="J48"/>
+      <c r="K48"/>
+      <c r="L48"/>
+      <c r="M48"/>
+      <c r="N48"/>
+      <c r="O48"/>
+      <c r="P48"/>
+      <c r="Q48"/>
+      <c r="R48"/>
+      <c r="S48"/>
+      <c r="T48"/>
+      <c r="U48"/>
+      <c r="V48"/>
+      <c r="W48"/>
+      <c r="X48"/>
+      <c r="Y48"/>
+      <c r="Z48"/>
+      <c r="AA48"/>
+      <c r="AB48"/>
+      <c r="AC48"/>
+      <c r="AD48"/>
+      <c r="AE48"/>
+      <c r="AF48"/>
+      <c r="AG48"/>
+      <c r="AH48"/>
+      <c r="AI48"/>
+      <c r="AJ48"/>
+      <c r="AK48"/>
+      <c r="AL48"/>
+      <c r="AM48"/>
+      <c r="AN48"/>
+      <c r="AO48"/>
+      <c r="AP48"/>
+      <c r="AQ48"/>
+    </row>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="84" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="85" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="86" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="87" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="88" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="89" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="90" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="91" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="92" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="93" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="94" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A5:H5"/>
+  <mergeCells count="13">
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>